<commit_message>
Regenerated deliverable supplement and gate artifact from the final code
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AhzzzJvfv5ysCRfLvXou8X
</commit_message>
<xml_diff>
--- a/nfl/dfs/salaries/DK_WEEK3_DELIVERABLE_SUPPLEMENT.xlsx
+++ b/nfl/dfs/salaries/DK_WEEK3_DELIVERABLE_SUPPLEMENT.xlsx
@@ -1723,7 +1723,7 @@
         </is>
       </c>
       <c r="D2">
-        <v>2.7</v>
+        <v>2.91</v>
       </c>
       <c r="E2">
         <v>336</v>
@@ -1751,7 +1751,7 @@
         </is>
       </c>
       <c r="D3">
-        <v>2.59</v>
+        <v>2.79</v>
       </c>
       <c r="E3">
         <v>336</v>
@@ -1779,7 +1779,7 @@
         </is>
       </c>
       <c r="D4">
-        <v>2.57</v>
+        <v>2.77</v>
       </c>
       <c r="E4">
         <v>336</v>
@@ -1807,7 +1807,7 @@
         </is>
       </c>
       <c r="D5">
-        <v>2.52</v>
+        <v>2.73</v>
       </c>
       <c r="E5">
         <v>720</v>
@@ -1835,7 +1835,7 @@
         </is>
       </c>
       <c r="D6">
-        <v>0.77</v>
+        <v>0.98</v>
       </c>
       <c r="E6">
         <v>336</v>
@@ -1863,7 +1863,7 @@
         </is>
       </c>
       <c r="D7">
-        <v>0.96</v>
+        <v>1.16</v>
       </c>
       <c r="E7">
         <v>336</v>
@@ -1891,7 +1891,7 @@
         </is>
       </c>
       <c r="D8">
-        <v>0.74</v>
+        <v>0.95</v>
       </c>
       <c r="E8">
         <v>336</v>
@@ -1919,7 +1919,7 @@
         </is>
       </c>
       <c r="D9">
-        <v>0.64</v>
+        <v>0.84</v>
       </c>
       <c r="E9">
         <v>336</v>
@@ -1947,7 +1947,7 @@
         </is>
       </c>
       <c r="D10">
-        <v>1.01</v>
+        <v>1.22</v>
       </c>
       <c r="E10">
         <v>720</v>
@@ -1975,7 +1975,7 @@
         </is>
       </c>
       <c r="D11">
-        <v>0.71</v>
+        <v>0.92</v>
       </c>
       <c r="E11">
         <v>168</v>
@@ -2003,7 +2003,7 @@
         </is>
       </c>
       <c r="D12">
-        <v>1.98</v>
+        <v>2.19</v>
       </c>
       <c r="E12">
         <v>36</v>
@@ -2031,7 +2031,7 @@
         </is>
       </c>
       <c r="D13">
-        <v>11.64</v>
+        <v>11.85</v>
       </c>
       <c r="E13">
         <v>6</v>
@@ -2059,7 +2059,7 @@
         </is>
       </c>
       <c r="D14">
-        <v>1.05</v>
+        <v>1.26</v>
       </c>
       <c r="E14">
         <v>36</v>
@@ -2087,7 +2087,7 @@
         </is>
       </c>
       <c r="D15">
-        <v>0.12</v>
+        <v>0.33</v>
       </c>
       <c r="E15">
         <v>24</v>
@@ -2209,7 +2209,7 @@
         </is>
       </c>
       <c r="B6">
-        <v>1790568374</v>
+        <v>1790569118</v>
       </c>
     </row>
     <row r="7">

</xml_diff>

<commit_message>
Regenerate field, portfolio and deliverable against the corrected projections
The readiness board flagged field.model and portfolio.contest as FRESH_BUT_BEHIND_ITS_INPUTS after the
projection rebuild, which is that check doing its job on a real case rather than a synthetic one.

Portfolio result holds on the corrected projections: P(at least one entry in the top 1%) 0.7700 for
joint selection against independent, 1.54x, for 1.68 projected points per entry. The method still wins
at every field setting tested (0.17 to 0.34 absolute) while the specific 48 entries still overlap the
base by only 0.48 to 0.58, so the split verdict is unchanged: method usable, entries not determined.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AhzzzJvfv5ysCRfLvXou8X
</commit_message>
<xml_diff>
--- a/nfl/dfs/salaries/DK_WEEK3_DELIVERABLE_SUPPLEMENT.xlsx
+++ b/nfl/dfs/salaries/DK_WEEK3_DELIVERABLE_SUPPLEMENT.xlsx
@@ -69,36 +69,36 @@
         </is>
       </c>
       <c r="B2">
-        <v>0.5135</v>
+        <v>0.4823</v>
       </c>
       <c r="C2">
-        <v>0.5186</v>
+        <v>0.4914</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Kenneth Walker III</t>
+          <t xml:space="preserve">Amon-Ra St. Brown</t>
         </is>
       </c>
       <c r="B3">
-        <v>0.4158</v>
+        <v>0.3844</v>
       </c>
       <c r="C3">
-        <v>0.4144</v>
+        <v>0.3828</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Jaxon Smith-Njigba</t>
+          <t xml:space="preserve">Jahmyr Gibbs</t>
         </is>
       </c>
       <c r="B4">
-        <v>0.3686</v>
+        <v>0.3769</v>
       </c>
       <c r="C4">
-        <v>0.3721</v>
+        <v>0.3872</v>
       </c>
     </row>
     <row r="5">
@@ -108,62 +108,62 @@
         </is>
       </c>
       <c r="B5">
-        <v>0.3589</v>
+        <v>0.3588</v>
       </c>
       <c r="C5">
-        <v>0.3639</v>
+        <v>0.3643</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Amon-Ra St. Brown</t>
+          <t xml:space="preserve">Jaxon Smith-Njigba</t>
         </is>
       </c>
       <c r="B6">
-        <v>0.3552</v>
+        <v>0.3585</v>
       </c>
       <c r="C6">
-        <v>0.3528</v>
+        <v>0.3558</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t xml:space="preserve">Garrett Wilson</t>
+          <t xml:space="preserve">Kenneth Walker III</t>
         </is>
       </c>
       <c r="B7">
-        <v>0.3002</v>
+        <v>0.3579</v>
       </c>
       <c r="C7">
-        <v>0.3041</v>
+        <v>0.3606</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Jahmyr Gibbs</t>
+          <t xml:space="preserve">Travis Kelce</t>
         </is>
       </c>
       <c r="B8">
-        <v>0.2949</v>
+        <v>0.3204</v>
       </c>
       <c r="C8">
-        <v>0.2986</v>
+        <v>0.3168</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Travis Kelce</t>
+          <t xml:space="preserve">Garrett Wilson</t>
         </is>
       </c>
       <c r="B9">
-        <v>0.2783</v>
+        <v>0.2933</v>
       </c>
       <c r="C9">
-        <v>0.2783</v>
+        <v>0.2963</v>
       </c>
     </row>
     <row r="10">
@@ -173,62 +173,62 @@
         </is>
       </c>
       <c r="B10">
-        <v>0.2111</v>
+        <v>0.1989</v>
       </c>
       <c r="C10">
-        <v>0.2123</v>
+        <v>0.2013</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t xml:space="preserve">Josh Allen</t>
+          <t xml:space="preserve">Parker Washington</t>
         </is>
       </c>
       <c r="B11">
-        <v>0.1867</v>
+        <v>0.1961</v>
       </c>
       <c r="C11">
-        <v>0.1883</v>
+        <v>0.1964</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Breece Hall</t>
+          <t xml:space="preserve">Josh Allen</t>
         </is>
       </c>
       <c r="B12">
-        <v>0.1853</v>
+        <v>0.1908</v>
       </c>
       <c r="C12">
-        <v>0.1931</v>
+        <v>0.1875</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t xml:space="preserve">Dalton Kincaid</t>
+          <t xml:space="preserve">Breece Hall</t>
         </is>
       </c>
       <c r="B13">
-        <v>0.1731</v>
+        <v>0.1892</v>
       </c>
       <c r="C13">
-        <v>0.1725</v>
+        <v>0.1949</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t xml:space="preserve">Parker Washington</t>
+          <t xml:space="preserve">Dalton Kincaid</t>
         </is>
       </c>
       <c r="B14">
-        <v>0.166</v>
+        <v>0.1828</v>
       </c>
       <c r="C14">
-        <v>0.1628</v>
+        <v>0.1775</v>
       </c>
     </row>
     <row r="15">
@@ -238,23 +238,23 @@
         </is>
       </c>
       <c r="B15">
-        <v>0.1528</v>
+        <v>0.1577</v>
       </c>
       <c r="C15">
-        <v>0.1594</v>
+        <v>0.1644</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t xml:space="preserve">Jonathan Taylor</t>
+          <t xml:space="preserve">Sam LaPorta</t>
         </is>
       </c>
       <c r="B16">
-        <v>0.15</v>
+        <v>0.1185</v>
       </c>
       <c r="C16">
-        <v>0.1549</v>
+        <v>0.1213</v>
       </c>
     </row>
     <row r="17"/>
@@ -350,13 +350,13 @@
         <v>1</v>
       </c>
       <c r="B2">
-        <v>49700</v>
+        <v>49900</v>
       </c>
       <c r="C2">
-        <v>162.5363</v>
+        <v>160.3805</v>
       </c>
       <c r="D2">
-        <v>158.8048</v>
+        <v>157.5746</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
@@ -365,7 +365,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Patrick Mahomes | Kenneth Walker III | De'Von Achane | Garrett Wilson | Parker Washington | Ladd McConkey | Travis Kelce | Dalton Schultz | Steelers</t>
+          <t xml:space="preserve">Patrick Mahomes | Kenneth Walker III | Breece Hall | Jaylen Warren | Garrett Wilson | Parker Washington | Tre' Harris | Dalton Schultz | Seahawks</t>
         </is>
       </c>
     </row>
@@ -374,22 +374,22 @@
         <v>2</v>
       </c>
       <c r="B3">
-        <v>49800</v>
+        <v>49600</v>
       </c>
       <c r="C3">
-        <v>163.4631</v>
+        <v>161.6316</v>
       </c>
       <c r="D3">
-        <v>157.3381</v>
+        <v>155.5882</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t xml:space="preserve">VALUE_FRONTIER</t>
+          <t xml:space="preserve">BEST_WITH_RB</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Patrick Mahomes | Kenneth Walker III | Breece Hall | Jaylen Warren | Garrett Wilson | Ladd McConkey | Tre' Harris | Dalton Schultz | Seahawks</t>
+          <t xml:space="preserve">Patrick Mahomes | Kenneth Walker III | De'Von Achane | Amon-Ra St. Brown | Garrett Wilson | Tre' Harris | Travis Kelce | Dalton Schultz | Steelers</t>
         </is>
       </c>
     </row>
@@ -398,13 +398,13 @@
         <v>3</v>
       </c>
       <c r="B4">
-        <v>50000</v>
+        <v>49800</v>
       </c>
       <c r="C4">
-        <v>163.3098</v>
+        <v>161.9198</v>
       </c>
       <c r="D4">
-        <v>155.7187</v>
+        <v>154.3331</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
@@ -413,7 +413,7 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Marcus Mariota | Kenneth Walker III | Breece Hall | Amon-Ra St. Brown | Garrett Wilson | Ladd McConkey | Travis Kelce | Dalton Schultz | Bengals</t>
+          <t xml:space="preserve">Josh Allen | Kenneth Walker III | Breece Hall | Garrett Wilson | Ladd McConkey | Tre' Harris | Travis Kelce | Dalton Schultz | Texans</t>
         </is>
       </c>
     </row>
@@ -422,13 +422,13 @@
         <v>4</v>
       </c>
       <c r="B5">
-        <v>49500</v>
+        <v>50000</v>
       </c>
       <c r="C5">
-        <v>162.1901</v>
+        <v>160.7034</v>
       </c>
       <c r="D5">
-        <v>151.855</v>
+        <v>154.6852</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
@@ -437,7 +437,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Deshaun Watson | Kenneth Walker III | Breece Hall | Jaxon Smith-Njigba | Garrett Wilson | Michael Pittman Jr. | Travis Kelce | Dalton Schultz | Steelers</t>
+          <t xml:space="preserve">C.J. Stroud | Kenneth Walker III | Breece Hall | Jaylen Warren | Amon-Ra St. Brown | Garrett Wilson | Tre' Harris | Dalton Schultz | Steelers</t>
         </is>
       </c>
     </row>
@@ -446,22 +446,22 @@
         <v>5</v>
       </c>
       <c r="B6">
-        <v>49700</v>
+        <v>50000</v>
       </c>
       <c r="C6">
-        <v>162.6074</v>
+        <v>162.0642</v>
       </c>
       <c r="D6">
-        <v>153.5436</v>
+        <v>151.6626</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t xml:space="preserve">BEST_WITH_TE</t>
+          <t xml:space="preserve">VALUE_FRONTIER</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Patrick Mahomes | Kenneth Walker III | Breece Hall | Amon-Ra St. Brown | Garrett Wilson | Tre' Harris | Isaiah Likely | Dalton Schultz | Steelers</t>
+          <t xml:space="preserve">Patrick Mahomes | Jahmyr Gibbs | Kenneth Walker III | Garrett Wilson | Parker Washington | Jaylin Noel | Travis Kelce | Dalton Schultz | Panthers</t>
         </is>
       </c>
     </row>
@@ -473,10 +473,10 @@
         <v>49800</v>
       </c>
       <c r="C7">
-        <v>162.7914</v>
+        <v>161.0842</v>
       </c>
       <c r="D7">
-        <v>155.0343</v>
+        <v>152.555</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -485,7 +485,7 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t xml:space="preserve">Josh Allen | Kenneth Walker III | Jaylen Warren | Garrett Wilson | Parker Washington | Tre' Harris | Travis Kelce | Dalton Schultz | Seahawks</t>
+          <t xml:space="preserve">Patrick Mahomes | Jahmyr Gibbs | Kenneth Walker III | Parker Washington | Ladd McConkey | Tre' Harris | Travis Kelce | Dalton Schultz | Bengals</t>
         </is>
       </c>
     </row>
@@ -494,13 +494,13 @@
         <v>7</v>
       </c>
       <c r="B8">
-        <v>49700</v>
+        <v>49800</v>
       </c>
       <c r="C8">
-        <v>163.2173</v>
+        <v>160.8528</v>
       </c>
       <c r="D8">
-        <v>149.7265</v>
+        <v>151.2266</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -509,7 +509,7 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Josh Allen | Jahmyr Gibbs | Kenneth Walker III | Garrett Wilson | Tre' Harris | Jaylin Noel | Travis Kelce | Dalton Schultz | Panthers</t>
+          <t xml:space="preserve">Josh Allen | Kenneth Walker III | Breece Hall | Garrett Wilson | Ladd McConkey | Michael Pittman Jr. | Travis Kelce | Dalton Schultz | Titans</t>
         </is>
       </c>
     </row>
@@ -521,10 +521,10 @@
         <v>50000</v>
       </c>
       <c r="C9">
-        <v>162.8921</v>
+        <v>160.9235</v>
       </c>
       <c r="D9">
-        <v>150.2944</v>
+        <v>151.1031</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
@@ -533,7 +533,7 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Patrick Mahomes | Kenneth Walker III | Breece Hall | Amon-Ra St. Brown | Parker Washington | Jaylin Noel | Travis Kelce | Dalton Schultz | Seahawks</t>
+          <t xml:space="preserve">Josh Allen | Jahmyr Gibbs | Jaylen Warren | Garrett Wilson | Ladd McConkey | Tre' Harris | Travis Kelce | Dalton Schultz | Steelers</t>
         </is>
       </c>
     </row>
@@ -542,22 +542,22 @@
         <v>9</v>
       </c>
       <c r="B10">
-        <v>49600</v>
+        <v>49900</v>
       </c>
       <c r="C10">
-        <v>162.7671</v>
+        <v>160.7435</v>
       </c>
       <c r="D10">
-        <v>151.4148</v>
+        <v>155.5758</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t xml:space="preserve">BEST_WITH_QB</t>
+          <t xml:space="preserve">VALUE_FRONTIER</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Jared Goff | Kenneth Walker III | Breece Hall | Amon-Ra St. Brown | Garrett Wilson | Tre' Harris | Travis Kelce | Dalton Schultz | Steelers</t>
+          <t xml:space="preserve">Deshaun Watson | Kenneth Walker III | Breece Hall | Amon-Ra St. Brown | Garrett Wilson | Parker Washington | Travis Kelce | Dalton Schultz | Browns</t>
         </is>
       </c>
     </row>
@@ -566,22 +566,22 @@
         <v>10</v>
       </c>
       <c r="B11">
-        <v>50000</v>
+        <v>49700</v>
       </c>
       <c r="C11">
-        <v>159.1739</v>
+        <v>159.9127</v>
       </c>
       <c r="D11">
-        <v>150.5445</v>
+        <v>153.1904</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t xml:space="preserve">BEST_WITH_RB</t>
+          <t xml:space="preserve">BEST_WITH_QB</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t xml:space="preserve">Josh Allen | Kenneth Walker III | Breece Hall | Quinshon Judkins | Garrett Wilson | Ladd McConkey | Jaylin Noel | Dalton Schultz | Steelers</t>
+          <t xml:space="preserve">Jameis Winston | Jahmyr Gibbs | Kenneth Walker III | Amon-Ra St. Brown | Garrett Wilson | Tre' Harris | Travis Kelce | Dalton Schultz | Steelers</t>
         </is>
       </c>
     </row>
@@ -590,22 +590,22 @@
         <v>11</v>
       </c>
       <c r="B12">
-        <v>50000</v>
+        <v>49900</v>
       </c>
       <c r="C12">
-        <v>161.8097</v>
+        <v>160.7878</v>
       </c>
       <c r="D12">
-        <v>155.6203</v>
+        <v>152.3818</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t xml:space="preserve">BEST_WITH_QB</t>
+          <t xml:space="preserve">VALUE_FRONTIER</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Jameis Winston | Kenneth Walker III | Breece Hall | Jaxon Smith-Njigba | Garrett Wilson | Ladd McConkey | Travis Kelce | Dalton Schultz | Steelers</t>
+          <t xml:space="preserve">Josh Allen | Breece Hall | Jaylen Warren | Amon-Ra St. Brown | Garrett Wilson | Tre' Harris | Travis Kelce | Dalton Schultz | Panthers</t>
         </is>
       </c>
     </row>
@@ -614,13 +614,13 @@
         <v>12</v>
       </c>
       <c r="B13">
-        <v>49900</v>
+        <v>50000</v>
       </c>
       <c r="C13">
-        <v>162.6742</v>
+        <v>160.3729</v>
       </c>
       <c r="D13">
-        <v>150.9844</v>
+        <v>150.551</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
@@ -629,7 +629,7 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t xml:space="preserve">Josh Allen | Kenneth Walker III | James Cook III | Garrett Wilson | Parker Washington | Tre' Harris | Travis Kelce | Dalton Schultz | Steelers</t>
+          <t xml:space="preserve">Patrick Mahomes | Kenneth Walker III | Breece Hall | Jaxon Smith-Njigba | Ladd McConkey | Tre' Harris | Travis Kelce | Dalton Schultz | Jaguars</t>
         </is>
       </c>
     </row>
@@ -641,10 +641,10 @@
         <v>50000</v>
       </c>
       <c r="C14">
-        <v>162.6667</v>
+        <v>160.802</v>
       </c>
       <c r="D14">
-        <v>150.5654</v>
+        <v>152.0121</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
@@ -653,7 +653,7 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t xml:space="preserve">Josh Allen | Kenneth Walker III | Breece Hall | Parker Washington | Ladd McConkey | Michael Pittman Jr. | Travis Kelce | Dalton Schultz | Bengals</t>
+          <t xml:space="preserve">Deshaun Watson | Jahmyr Gibbs | Kenneth Walker III | Breece Hall | Garrett Wilson | Ladd McConkey | Jaylin Noel | Dalton Schultz | Steelers</t>
         </is>
       </c>
     </row>
@@ -665,19 +665,19 @@
         <v>50000</v>
       </c>
       <c r="C15">
-        <v>162.3385</v>
+        <v>160.0912</v>
       </c>
       <c r="D15">
-        <v>150.4268</v>
+        <v>152.9676</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t xml:space="preserve">VALUE_FRONTIER</t>
+          <t xml:space="preserve">BEST_WITH_TE</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t xml:space="preserve">Patrick Mahomes | Kenneth Walker III | Breece Hall | Jaylen Warren | Rashee Rice | Garrett Wilson | Michael Pittman Jr. | Dalton Schultz | Steelers</t>
+          <t xml:space="preserve">Patrick Mahomes | Kenneth Walker III | Breece Hall | Amon-Ra St. Brown | Garrett Wilson | Tre' Harris | Dalton Schultz | Hunter Henry | Seahawks</t>
         </is>
       </c>
     </row>
@@ -686,13 +686,13 @@
         <v>15</v>
       </c>
       <c r="B16">
-        <v>50000</v>
+        <v>49900</v>
       </c>
       <c r="C16">
-        <v>162.9604</v>
+        <v>160.9309</v>
       </c>
       <c r="D16">
-        <v>151.6086</v>
+        <v>147.9515</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
@@ -701,7 +701,7 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t xml:space="preserve">Josh Allen | Kenneth Walker III | Jaylen Warren | Amon-Ra St. Brown | Garrett Wilson | Jaylin Noel | Travis Kelce | Dalton Schultz | Titans</t>
+          <t xml:space="preserve">Josh Allen | Kenneth Walker III | Breece Hall | Amon-Ra St. Brown | Michael Pittman Jr. | Tre' Harris | Travis Kelce | Dalton Schultz | Jaguars</t>
         </is>
       </c>
     </row>
@@ -710,13 +710,13 @@
         <v>16</v>
       </c>
       <c r="B17">
-        <v>49800</v>
+        <v>50000</v>
       </c>
       <c r="C17">
-        <v>162.8204</v>
+        <v>160.4449</v>
       </c>
       <c r="D17">
-        <v>152.8991</v>
+        <v>150.4551</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
@@ -725,7 +725,7 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t xml:space="preserve">Patrick Mahomes | Jahmyr Gibbs | Kenneth Walker III | Breece Hall | Garrett Wilson | Tre' Harris | Jaylin Noel | Dalton Schultz | Panthers</t>
+          <t xml:space="preserve">Patrick Mahomes | Kenneth Walker III | Breece Hall | Jaxon Smith-Njigba | Garrett Wilson | Tre' Harris | Sam LaPorta | Dalton Schultz | Steelers</t>
         </is>
       </c>
     </row>
@@ -734,13 +734,13 @@
         <v>17</v>
       </c>
       <c r="B18">
-        <v>49700</v>
+        <v>50000</v>
       </c>
       <c r="C18">
-        <v>162.5353</v>
+        <v>158.4838</v>
       </c>
       <c r="D18">
-        <v>153.6231</v>
+        <v>143.3149</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
@@ -749,7 +749,7 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t xml:space="preserve">Patrick Mahomes | Kenneth Walker III | Chase Brown | Amon-Ra St. Brown | Garrett Wilson | Tre' Harris | Travis Kelce | Dalton Schultz | Steelers</t>
+          <t xml:space="preserve">Patrick Mahomes | Jonathan Taylor | Kenneth Walker III | Amon-Ra St. Brown | Ladd McConkey | Jaylin Noel | Travis Kelce | Dalton Schultz | Steelers</t>
         </is>
       </c>
     </row>
@@ -758,22 +758,22 @@
         <v>18</v>
       </c>
       <c r="B19">
-        <v>49900</v>
+        <v>50000</v>
       </c>
       <c r="C19">
-        <v>162.4472</v>
+        <v>159.621</v>
       </c>
       <c r="D19">
-        <v>153.469</v>
+        <v>147.3436</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t xml:space="preserve">VALUE_FRONTIER</t>
+          <t xml:space="preserve">BEST_WITH_TE</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t xml:space="preserve">Deshaun Watson | Kenneth Walker III | Breece Hall | Amon-Ra St. Brown | Garrett Wilson | Michael Pittman Jr. | Travis Kelce | Dalton Schultz | Seahawks</t>
+          <t xml:space="preserve">Josh Allen | Kenneth Walker III | Breece Hall | Garrett Wilson | Ladd McConkey | Jaylin Noel | Dalton Kincaid | Dalton Schultz | Steelers</t>
         </is>
       </c>
     </row>
@@ -782,13 +782,13 @@
         <v>19</v>
       </c>
       <c r="B20">
-        <v>50000</v>
+        <v>49800</v>
       </c>
       <c r="C20">
-        <v>162.2927</v>
+        <v>160.6504</v>
       </c>
       <c r="D20">
-        <v>154.1282</v>
+        <v>146.8705</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
@@ -797,7 +797,7 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t xml:space="preserve">Patrick Mahomes | Kenneth Walker III | Breece Hall | Amon-Ra St. Brown | Garrett Wilson | Tre' Harris | Dalton Schultz | Hunter Henry | Seahawks</t>
+          <t xml:space="preserve">Patrick Mahomes | Jahmyr Gibbs | Breece Hall | Garrett Wilson | Parker Washington | Michael Pittman Jr. | Travis Kelce | Dalton Schultz | Steelers</t>
         </is>
       </c>
     </row>
@@ -806,22 +806,22 @@
         <v>20</v>
       </c>
       <c r="B21">
-        <v>49900</v>
+        <v>50000</v>
       </c>
       <c r="C21">
-        <v>162.1768</v>
+        <v>159.8654</v>
       </c>
       <c r="D21">
-        <v>150.1345</v>
+        <v>151.7472</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t xml:space="preserve">VALUE_FRONTIER</t>
+          <t xml:space="preserve">BEST_WITH_WR</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t xml:space="preserve">Josh Allen | Kenneth Walker III | Breece Hall | Jaylen Warren | Parker Washington | Ladd McConkey | Jaylin Noel | Dalton Schultz | Steelers</t>
+          <t xml:space="preserve">Patrick Mahomes | Kenneth Walker III | Jaylen Warren | Amon-Ra St. Brown | Garrett Wilson | Romeo Doubs | Travis Kelce | Dalton Schultz | Steelers</t>
         </is>
       </c>
     </row>
@@ -830,13 +830,13 @@
         <v>21</v>
       </c>
       <c r="B22">
-        <v>50000</v>
+        <v>49600</v>
       </c>
       <c r="C22">
-        <v>164.1895</v>
+        <v>162.0308</v>
       </c>
       <c r="D22">
-        <v>154.3442</v>
+        <v>156.1281</v>
       </c>
       <c r="E22" t="inlineStr">
         <is>
@@ -845,7 +845,7 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t xml:space="preserve">Patrick Mahomes | Jahmyr Gibbs | Kenneth Walker III | Garrett Wilson | Parker Washington | Tre' Harris | Travis Kelce | Dalton Schultz | Steelers</t>
+          <t xml:space="preserve">Josh Allen | Kenneth Walker III | Breece Hall | Garrett Wilson | Parker Washington | Tre' Harris | Travis Kelce | Dalton Schultz | Jaguars</t>
         </is>
       </c>
     </row>
@@ -854,13 +854,13 @@
         <v>22</v>
       </c>
       <c r="B23">
-        <v>49800</v>
+        <v>50000</v>
       </c>
       <c r="C23">
-        <v>163.0641</v>
+        <v>161.187</v>
       </c>
       <c r="D23">
-        <v>152.6097</v>
+        <v>155.0313</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
@@ -869,7 +869,7 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t xml:space="preserve">Patrick Mahomes | Kenneth Walker III | Jaylen Warren | Amon-Ra St. Brown | Garrett Wilson | Michael Pittman Jr. | Travis Kelce | Dalton Schultz | Bengals</t>
+          <t xml:space="preserve">Patrick Mahomes | Kenneth Walker III | Jaylen Warren | Garrett Wilson | Parker Washington | Ladd McConkey | Travis Kelce | Dalton Schultz | Seahawks</t>
         </is>
       </c>
     </row>
@@ -881,10 +881,10 @@
         <v>50000</v>
       </c>
       <c r="C24">
-        <v>162.8801</v>
+        <v>160.6156</v>
       </c>
       <c r="D24">
-        <v>148.4065</v>
+        <v>154.5692</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
@@ -893,7 +893,7 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t xml:space="preserve">Josh Allen | Kenneth Walker III | Breece Hall | Garrett Wilson | Ladd McConkey | Jaylin Noel | Dalton Kincaid | Dalton Schultz | Steelers</t>
+          <t xml:space="preserve">C.J. Stroud | Kenneth Walker III | Breece Hall | Garrett Wilson | Parker Washington | Ladd McConkey | Travis Kelce | Dalton Schultz | Seahawks</t>
         </is>
       </c>
     </row>
@@ -902,13 +902,13 @@
         <v>24</v>
       </c>
       <c r="B25">
-        <v>49800</v>
+        <v>50000</v>
       </c>
       <c r="C25">
-        <v>162.5717</v>
+        <v>160.3564</v>
       </c>
       <c r="D25">
-        <v>153.3608</v>
+        <v>145.7147</v>
       </c>
       <c r="E25" t="inlineStr">
         <is>
@@ -917,7 +917,7 @@
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t xml:space="preserve">C.J. Stroud | Kenneth Walker III | Breece Hall | Jaxon Smith-Njigba | Garrett Wilson | Tre' Harris | Travis Kelce | Dalton Schultz | Panthers</t>
+          <t xml:space="preserve">Deshaun Watson | Kenneth Walker III | Breece Hall | Jaxon Smith-Njigba | Amon-Ra St. Brown | Jaylin Noel | Travis Kelce | Dalton Schultz | Steelers</t>
         </is>
       </c>
     </row>
@@ -926,22 +926,22 @@
         <v>25</v>
       </c>
       <c r="B26">
-        <v>49800</v>
+        <v>50000</v>
       </c>
       <c r="C26">
-        <v>162.495</v>
+        <v>160.095</v>
       </c>
       <c r="D26">
-        <v>151.2777</v>
+        <v>152.2921</v>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t xml:space="preserve">VALUE_FRONTIER</t>
+          <t xml:space="preserve">BEST_WITH_WR</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t xml:space="preserve">Patrick Mahomes | Jahmyr Gibbs | Kenneth Walker III | Garrett Wilson | Ladd McConkey | Jaylin Noel | Travis Kelce | Dalton Schultz | Jaguars</t>
+          <t xml:space="preserve">Patrick Mahomes | Jahmyr Gibbs | Kenneth Walker III | Garrett Wilson | Tetairoa McMillan | Tre' Harris | Travis Kelce | Dalton Schultz | Steelers</t>
         </is>
       </c>
     </row>
@@ -950,13 +950,13 @@
         <v>26</v>
       </c>
       <c r="B27">
-        <v>50000</v>
+        <v>49800</v>
       </c>
       <c r="C27">
-        <v>162.1987</v>
+        <v>161.8645</v>
       </c>
       <c r="D27">
-        <v>146.7805</v>
+        <v>150.3276</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
@@ -965,7 +965,7 @@
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t xml:space="preserve">Josh Allen | Kenneth Walker III | Breece Hall | Rashee Rice | Garrett Wilson | Tre' Harris | Jaylin Noel | Dalton Schultz | Seahawks</t>
+          <t xml:space="preserve">Patrick Mahomes | Jahmyr Gibbs | Kenneth Walker III | Garrett Wilson | Ladd McConkey | Jaylin Noel | Travis Kelce | Dalton Schultz | Bengals</t>
         </is>
       </c>
     </row>
@@ -977,19 +977,19 @@
         <v>50000</v>
       </c>
       <c r="C28">
-        <v>162.5502</v>
+        <v>161.5618</v>
       </c>
       <c r="D28">
-        <v>149.0815</v>
+        <v>148.019</v>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t xml:space="preserve">BEST_WITH_RB</t>
+          <t xml:space="preserve">VALUE_FRONTIER</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t xml:space="preserve">Josh Allen | Kenneth Walker III | Rhamondre Stevenson | Amon-Ra St. Brown | Garrett Wilson | Jaylin Noel | Travis Kelce | Dalton Schultz | Steelers</t>
+          <t xml:space="preserve">Josh Allen | Kenneth Walker III | Jaylen Warren | Amon-Ra St. Brown | Parker Washington | Jaylin Noel | Travis Kelce | Dalton Schultz | Steelers</t>
         </is>
       </c>
     </row>
@@ -1001,10 +1001,10 @@
         <v>49900</v>
       </c>
       <c r="C29">
-        <v>163.7737</v>
+        <v>160.954</v>
       </c>
       <c r="D29">
-        <v>151.7581</v>
+        <v>145.3573</v>
       </c>
       <c r="E29" t="inlineStr">
         <is>
@@ -1013,7 +1013,7 @@
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t xml:space="preserve">Patrick Mahomes | Kenneth Walker III | Breece Hall | Jaxon Smith-Njigba | Parker Washington | Tre' Harris | Travis Kelce | Dalton Schultz | Steelers</t>
+          <t xml:space="preserve">Patrick Mahomes | Jahmyr Gibbs | Kenneth Walker III | Jaxon Smith-Njigba | Tre' Harris | Jaylin Noel | Travis Kelce | Dalton Schultz | Steelers</t>
         </is>
       </c>
     </row>
@@ -1022,13 +1022,13 @@
         <v>29</v>
       </c>
       <c r="B30">
-        <v>49500</v>
+        <v>50000</v>
       </c>
       <c r="C30">
-        <v>162.5956</v>
+        <v>160.8618</v>
       </c>
       <c r="D30">
-        <v>147.2054</v>
+        <v>149.4332</v>
       </c>
       <c r="E30" t="inlineStr">
         <is>
@@ -1037,7 +1037,7 @@
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t xml:space="preserve">Josh Allen | Kenneth Walker III | Breece Hall | Jaxon Smith-Njigba | Tre' Harris | Jaylin Noel | Travis Kelce | Dalton Schultz | Bengals</t>
+          <t xml:space="preserve">Josh Allen | Kenneth Walker III | Breece Hall | Parker Washington | Ladd McConkey | Michael Pittman Jr. | Travis Kelce | Dalton Schultz | Bengals</t>
         </is>
       </c>
     </row>
@@ -1046,13 +1046,13 @@
         <v>30</v>
       </c>
       <c r="B31">
-        <v>49900</v>
+        <v>50000</v>
       </c>
       <c r="C31">
-        <v>162.3945</v>
+        <v>160.6238</v>
       </c>
       <c r="D31">
-        <v>158.207</v>
+        <v>147.9297</v>
       </c>
       <c r="E31" t="inlineStr">
         <is>
@@ -1061,7 +1061,7 @@
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t xml:space="preserve">Patrick Mahomes | Kenneth Walker III | Breece Hall | Jaylen Warren | Garrett Wilson | Parker Washington | Tre' Harris | Dalton Schultz | Seahawks</t>
+          <t xml:space="preserve">C.J. Stroud | Jahmyr Gibbs | Kenneth Walker III | Garrett Wilson | Ladd McConkey | Michael Pittman Jr. | Travis Kelce | Dalton Schultz | Steelers</t>
         </is>
       </c>
     </row>
@@ -1073,10 +1073,10 @@
         <v>49700</v>
       </c>
       <c r="C32">
-        <v>162.3658</v>
+        <v>160.6028</v>
       </c>
       <c r="D32">
-        <v>153.4258</v>
+        <v>151.7811</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
@@ -1085,7 +1085,7 @@
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t xml:space="preserve">C.J. Stroud | Kenneth Walker III | Breece Hall | Jaxon Smith-Njigba | Garrett Wilson | Tre' Harris | Travis Kelce | Dalton Schultz | Bengals</t>
+          <t xml:space="preserve">Josh Allen | Breece Hall | Jaylen Warren | Garrett Wilson | Parker Washington | Ladd McConkey | Travis Kelce | Dalton Schultz | Steelers</t>
         </is>
       </c>
     </row>
@@ -1094,13 +1094,13 @@
         <v>32</v>
       </c>
       <c r="B33">
-        <v>49900</v>
+        <v>49800</v>
       </c>
       <c r="C33">
-        <v>162.2794</v>
+        <v>160.5819</v>
       </c>
       <c r="D33">
-        <v>154.1558</v>
+        <v>152.3193</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
@@ -1109,7 +1109,7 @@
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t xml:space="preserve">Josh Allen | Kenneth Walker III | Breece Hall | Jaylen Warren | Garrett Wilson | Ladd McConkey | Jaylin Noel | Dalton Schultz | Titans</t>
+          <t xml:space="preserve">Josh Allen | Breece Hall | Jaylen Warren | Amon-Ra St. Brown | Garrett Wilson | Tre' Harris | Travis Kelce | Dalton Schultz | Bengals</t>
         </is>
       </c>
     </row>
@@ -1118,22 +1118,22 @@
         <v>33</v>
       </c>
       <c r="B34">
-        <v>50000</v>
+        <v>49500</v>
       </c>
       <c r="C34">
-        <v>160.7397</v>
+        <v>160.553</v>
       </c>
       <c r="D34">
-        <v>153.1707</v>
+        <v>146.5198</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t xml:space="preserve">BEST_WITH_QB</t>
+          <t xml:space="preserve">VALUE_FRONTIER</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sam Darnold | Kenneth Walker III | Jaylen Warren | Amon-Ra St. Brown | Garrett Wilson | Ladd McConkey | Travis Kelce | Dalton Schultz | Steelers</t>
+          <t xml:space="preserve">Josh Allen | Jahmyr Gibbs | Breece Hall | Garrett Wilson | Michael Pittman Jr. | Tre' Harris | Travis Kelce | Dalton Schultz | Steelers</t>
         </is>
       </c>
     </row>
@@ -1142,22 +1142,22 @@
         <v>34</v>
       </c>
       <c r="B35">
-        <v>49700</v>
+        <v>49600</v>
       </c>
       <c r="C35">
-        <v>158.6256</v>
+        <v>162.798</v>
       </c>
       <c r="D35">
-        <v>151.0406</v>
+        <v>156.5606</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t xml:space="preserve">BEST_WITH_QB</t>
+          <t xml:space="preserve">VALUE_FRONTIER</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t xml:space="preserve">Aaron Rodgers | Kenneth Walker III | Breece Hall | Amon-Ra St. Brown | Garrett Wilson | Ladd McConkey | Tre' Harris | Dalton Schultz | Steelers</t>
+          <t xml:space="preserve">Josh Allen | Kenneth Walker III | Breece Hall | Garrett Wilson | Parker Washington | Tre' Harris | Travis Kelce | Dalton Schultz | Bengals</t>
         </is>
       </c>
     </row>
@@ -1166,22 +1166,22 @@
         <v>35</v>
       </c>
       <c r="B36">
-        <v>50000</v>
+        <v>49500</v>
       </c>
       <c r="C36">
-        <v>162.0446</v>
+        <v>162.586</v>
       </c>
       <c r="D36">
-        <v>152.4128</v>
+        <v>150.0189</v>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t xml:space="preserve">BEST_WITH_DST</t>
+          <t xml:space="preserve">VALUE_FRONTIER</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t xml:space="preserve">Josh Allen | Kenneth Walker III | Breece Hall | Garrett Wilson | Ladd McConkey | Jaylin Noel | Travis Kelce | Dalton Schultz | Chiefs</t>
+          <t xml:space="preserve">Patrick Mahomes | Kenneth Walker III | Breece Hall | Amon-Ra St. Brown | Garrett Wilson | Jaylin Noel | Travis Kelce | Dalton Schultz | Panthers</t>
         </is>
       </c>
     </row>
@@ -1190,13 +1190,13 @@
         <v>36</v>
       </c>
       <c r="B37">
-        <v>49700</v>
+        <v>50000</v>
       </c>
       <c r="C37">
-        <v>165.0051</v>
+        <v>162.3068</v>
       </c>
       <c r="D37">
-        <v>155.1735</v>
+        <v>151.4813</v>
       </c>
       <c r="E37" t="inlineStr">
         <is>
@@ -1205,7 +1205,7 @@
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t xml:space="preserve">Patrick Mahomes | Kenneth Walker III | Breece Hall | Amon-Ra St. Brown | Garrett Wilson | Tre' Harris | Travis Kelce | Dalton Schultz | Jaguars</t>
+          <t xml:space="preserve">Josh Allen | Kenneth Walker III | Breece Hall | Rashee Rice | Garrett Wilson | Tre' Harris | Travis Kelce | Dalton Schultz | Bengals</t>
         </is>
       </c>
     </row>
@@ -1217,10 +1217,10 @@
         <v>49500</v>
       </c>
       <c r="C38">
-        <v>164.8395</v>
+        <v>162.2817</v>
       </c>
       <c r="D38">
-        <v>152.5408</v>
+        <v>152.7547</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
@@ -1229,7 +1229,7 @@
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t xml:space="preserve">Patrick Mahomes | Kenneth Walker III | Breece Hall | Amon-Ra St. Brown | Garrett Wilson | Jaylin Noel | Travis Kelce | Dalton Schultz | Panthers</t>
+          <t xml:space="preserve">Patrick Mahomes | Kenneth Walker III | Breece Hall | Amon-Ra St. Brown | Garrett Wilson | Tre' Harris | Travis Kelce | Dalton Schultz | Patriots</t>
         </is>
       </c>
     </row>
@@ -1238,13 +1238,13 @@
         <v>38</v>
       </c>
       <c r="B39">
-        <v>50000</v>
+        <v>49900</v>
       </c>
       <c r="C39">
-        <v>164.1484</v>
+        <v>162.0233</v>
       </c>
       <c r="D39">
-        <v>155.292</v>
+        <v>153.9821</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
@@ -1253,7 +1253,7 @@
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t xml:space="preserve">Patrick Mahomes | Kenneth Walker III | Breece Hall | Jaxon Smith-Njigba | Garrett Wilson | Tre' Harris | Travis Kelce | Dalton Schultz | Browns</t>
+          <t xml:space="preserve">Patrick Mahomes | Kenneth Walker III | Jaylen Warren | Amon-Ra St. Brown | Garrett Wilson | Tre' Harris | Travis Kelce | Dalton Schultz | Seahawks</t>
         </is>
       </c>
     </row>
@@ -1262,13 +1262,13 @@
         <v>39</v>
       </c>
       <c r="B40">
-        <v>50000</v>
+        <v>49700</v>
       </c>
       <c r="C40">
-        <v>163.9745</v>
+        <v>161.9668</v>
       </c>
       <c r="D40">
-        <v>148.2609</v>
+        <v>151.3119</v>
       </c>
       <c r="E40" t="inlineStr">
         <is>
@@ -1277,7 +1277,7 @@
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t xml:space="preserve">Josh Allen | Kenneth Walker III | Breece Hall | Amon-Ra St. Brown | Michael Pittman Jr. | Tre' Harris | Travis Kelce | Dalton Schultz | Panthers</t>
+          <t xml:space="preserve">Josh Allen | Jahmyr Gibbs | Kenneth Walker III | Garrett Wilson | Tre' Harris | Jaylin Noel | Travis Kelce | Dalton Schultz | Panthers</t>
         </is>
       </c>
     </row>
@@ -1286,13 +1286,13 @@
         <v>40</v>
       </c>
       <c r="B41">
-        <v>49600</v>
+        <v>49900</v>
       </c>
       <c r="C41">
-        <v>163.9213</v>
+        <v>161.7661</v>
       </c>
       <c r="D41">
-        <v>151.2197</v>
+        <v>153.1259</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
@@ -1301,7 +1301,7 @@
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t xml:space="preserve">Patrick Mahomes | Kenneth Walker III | Jaylen Warren | Amon-Ra St. Brown | Garrett Wilson | Michael Pittman Jr. | Travis Kelce | Dalton Schultz | Steelers</t>
+          <t xml:space="preserve">Patrick Mahomes | Jahmyr Gibbs | Kenneth Walker III | Garrett Wilson | Ladd McConkey | Tre' Harris | Travis Kelce | Dalton Schultz | Patriots</t>
         </is>
       </c>
     </row>
@@ -1310,13 +1310,13 @@
         <v>41</v>
       </c>
       <c r="B42">
-        <v>50000</v>
+        <v>49900</v>
       </c>
       <c r="C42">
-        <v>163.9106</v>
+        <v>161.7567</v>
       </c>
       <c r="D42">
-        <v>153.8223</v>
+        <v>153.9868</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
@@ -1325,7 +1325,7 @@
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t xml:space="preserve">Patrick Mahomes | Kenneth Walker III | Breece Hall | Amon-Ra St. Brown | Garrett Wilson | Michael Pittman Jr. | Travis Kelce | Dalton Schultz | Titans</t>
+          <t xml:space="preserve">Marcus Mariota | Kenneth Walker III | Breece Hall | Amon-Ra St. Brown | Garrett Wilson | Parker Washington | Travis Kelce | Dalton Schultz | Steelers</t>
         </is>
       </c>
     </row>
@@ -1334,13 +1334,13 @@
         <v>42</v>
       </c>
       <c r="B43">
-        <v>49400</v>
+        <v>49900</v>
       </c>
       <c r="C43">
-        <v>163.6372</v>
+        <v>161.6981</v>
       </c>
       <c r="D43">
-        <v>150.5943</v>
+        <v>148.384</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
@@ -1349,7 +1349,7 @@
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t xml:space="preserve">Josh Allen | Kenneth Walker III | Jaylen Warren | Garrett Wilson | Ladd McConkey | Michael Pittman Jr. | Travis Kelce | Dalton Schultz | Steelers</t>
+          <t xml:space="preserve">Josh Allen | Kenneth Walker III | Breece Hall | Amon-Ra St. Brown | Michael Pittman Jr. | Tre' Harris | Travis Kelce | Dalton Schultz | Bengals</t>
         </is>
       </c>
     </row>
@@ -1358,13 +1358,13 @@
         <v>43</v>
       </c>
       <c r="B44">
-        <v>50000</v>
+        <v>49800</v>
       </c>
       <c r="C44">
-        <v>163.5295</v>
+        <v>161.5427</v>
       </c>
       <c r="D44">
-        <v>149.8911</v>
+        <v>149.8101</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
@@ -1373,7 +1373,7 @@
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t xml:space="preserve">Patrick Mahomes | Kenneth Walker III | Breece Hall | Jaylen Warren | Amon-Ra St. Brown | Ladd McConkey | Jaylin Noel | Dalton Schultz | Steelers</t>
+          <t xml:space="preserve">Patrick Mahomes | Breece Hall | Jaylen Warren | Amon-Ra St. Brown | Garrett Wilson | Ladd McConkey | Travis Kelce | Dalton Schultz | Steelers</t>
         </is>
       </c>
     </row>
@@ -1382,13 +1382,13 @@
         <v>44</v>
       </c>
       <c r="B45">
-        <v>49800</v>
+        <v>49900</v>
       </c>
       <c r="C45">
-        <v>163.5239</v>
+        <v>161.5365</v>
       </c>
       <c r="D45">
-        <v>149.1754</v>
+        <v>151.0826</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
@@ -1397,7 +1397,7 @@
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t xml:space="preserve">Josh Allen | Kenneth Walker III | Breece Hall | Parker Washington | Ladd McConkey | Michael Pittman Jr. | Travis Kelce | Dalton Schultz | Steelers</t>
+          <t xml:space="preserve">Patrick Mahomes | Breece Hall | Jaylen Warren | Amon-Ra St. Brown | Garrett Wilson | Parker Washington | Travis Kelce | Dalton Schultz | Steelers</t>
         </is>
       </c>
     </row>
@@ -1406,13 +1406,13 @@
         <v>45</v>
       </c>
       <c r="B46">
-        <v>50000</v>
+        <v>49200</v>
       </c>
       <c r="C46">
-        <v>163.2179</v>
+        <v>161.4464</v>
       </c>
       <c r="D46">
-        <v>151.7693</v>
+        <v>150.6548</v>
       </c>
       <c r="E46" t="inlineStr">
         <is>
@@ -1421,7 +1421,7 @@
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t xml:space="preserve">Patrick Mahomes | Kenneth Walker III | Breece Hall | Jaxon Smith-Njigba | Ladd McConkey | Tre' Harris | Travis Kelce | Dalton Schultz | Jaguars</t>
+          <t xml:space="preserve">Josh Allen | Kenneth Walker III | Breece Hall | Garrett Wilson | Ladd McConkey | Jaylin Noel | Travis Kelce | Dalton Schultz | Bengals</t>
         </is>
       </c>
     </row>
@@ -1430,13 +1430,13 @@
         <v>46</v>
       </c>
       <c r="B47">
-        <v>49600</v>
+        <v>49900</v>
       </c>
       <c r="C47">
-        <v>162.6831</v>
+        <v>161.2901</v>
       </c>
       <c r="D47">
-        <v>149.135</v>
+        <v>152.6175</v>
       </c>
       <c r="E47" t="inlineStr">
         <is>
@@ -1445,7 +1445,7 @@
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t xml:space="preserve">Josh Allen | Breece Hall | Jaylen Warren | Amon-Ra St. Brown | Garrett Wilson | Tre' Harris | Travis Kelce | Dalton Schultz | Steelers</t>
+          <t xml:space="preserve">Patrick Mahomes | Jahmyr Gibbs | Kenneth Walker III | Parker Washington | Ladd McConkey | Tre' Harris | Travis Kelce | Dalton Schultz | Panthers</t>
         </is>
       </c>
     </row>
@@ -1454,13 +1454,13 @@
         <v>47</v>
       </c>
       <c r="B48">
-        <v>49800</v>
+        <v>49900</v>
       </c>
       <c r="C48">
-        <v>162.608</v>
+        <v>161.1249</v>
       </c>
       <c r="D48">
-        <v>149.669</v>
+        <v>154.0495</v>
       </c>
       <c r="E48" t="inlineStr">
         <is>
@@ -1469,7 +1469,7 @@
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t xml:space="preserve">Josh Allen | Kenneth Walker III | Breece Hall | Parker Washington | Ladd McConkey | Jaylin Noel | Travis Kelce | Dalton Schultz | Seahawks</t>
+          <t xml:space="preserve">Patrick Mahomes | Kenneth Walker III | Breece Hall | Jaxon Smith-Njigba | Garrett Wilson | Tre' Harris | Travis Kelce | Dalton Schultz | Titans</t>
         </is>
       </c>
     </row>
@@ -1478,13 +1478,13 @@
         <v>48</v>
       </c>
       <c r="B49">
-        <v>50000</v>
+        <v>49800</v>
       </c>
       <c r="C49">
-        <v>162.5412</v>
+        <v>161.0834</v>
       </c>
       <c r="D49">
-        <v>152.8313</v>
+        <v>155.953</v>
       </c>
       <c r="E49" t="inlineStr">
         <is>
@@ -1493,7 +1493,7 @@
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t xml:space="preserve">Josh Allen | Kenneth Walker III | Jaylen Warren | Amon-Ra St. Brown | Garrett Wilson | Tre' Harris | Travis Kelce | Dalton Schultz | Jets</t>
+          <t xml:space="preserve">Josh Allen | Kenneth Walker III | Jaylen Warren | Garrett Wilson | Parker Washington | Tre' Harris | Travis Kelce | Dalton Schultz | Seahawks</t>
         </is>
       </c>
     </row>
@@ -1555,13 +1555,13 @@
         </is>
       </c>
       <c r="B2">
-        <v>0.4775</v>
+        <v>0.5</v>
       </c>
       <c r="C2">
-        <v>164.7832</v>
+        <v>162.7486</v>
       </c>
       <c r="D2">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="E2">
         <v>1.0</v>
@@ -1574,13 +1574,13 @@
         </is>
       </c>
       <c r="B3">
-        <v>0.7575</v>
+        <v>0.77</v>
       </c>
       <c r="C3">
-        <v>162.7496</v>
+        <v>161.0701</v>
       </c>
       <c r="D3">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="E3">
         <v>1.0</v>
@@ -1606,10 +1606,10 @@
         </is>
       </c>
       <c r="B6">
-        <v>0.9025</v>
+        <v>0.8875</v>
       </c>
       <c r="C6">
-        <v>0.7175</v>
+        <v>0.7225</v>
       </c>
       <c r="D6">
         <v>0.4792</v>
@@ -1623,13 +1623,13 @@
         </is>
       </c>
       <c r="B7">
-        <v>0.7175</v>
+        <v>0.7025</v>
       </c>
       <c r="C7">
-        <v>0.4025</v>
+        <v>0.3625</v>
       </c>
       <c r="D7">
-        <v>0.5208</v>
+        <v>0.5</v>
       </c>
       <c r="E7"/>
     </row>
@@ -1640,13 +1640,13 @@
         </is>
       </c>
       <c r="B8">
-        <v>0.8575</v>
+        <v>0.8775</v>
       </c>
       <c r="C8">
-        <v>0.605</v>
+        <v>0.635</v>
       </c>
       <c r="D8">
-        <v>0.4583</v>
+        <v>0.5833</v>
       </c>
       <c r="E8"/>
     </row>
@@ -1657,13 +1657,13 @@
         </is>
       </c>
       <c r="B9">
-        <v>0.755</v>
+        <v>0.73</v>
       </c>
       <c r="C9">
-        <v>0.49</v>
+        <v>0.4975</v>
       </c>
       <c r="D9">
-        <v>0.625</v>
+        <v>0.5625</v>
       </c>
       <c r="E9"/>
     </row>
@@ -1723,7 +1723,7 @@
         </is>
       </c>
       <c r="D2">
-        <v>2.91</v>
+        <v>12.67</v>
       </c>
       <c r="E2">
         <v>336</v>
@@ -1751,7 +1751,7 @@
         </is>
       </c>
       <c r="D3">
-        <v>2.79</v>
+        <v>12.55</v>
       </c>
       <c r="E3">
         <v>336</v>
@@ -1779,7 +1779,7 @@
         </is>
       </c>
       <c r="D4">
-        <v>2.77</v>
+        <v>12.53</v>
       </c>
       <c r="E4">
         <v>336</v>
@@ -1807,7 +1807,7 @@
         </is>
       </c>
       <c r="D5">
-        <v>2.73</v>
+        <v>12.49</v>
       </c>
       <c r="E5">
         <v>720</v>
@@ -1835,7 +1835,7 @@
         </is>
       </c>
       <c r="D6">
-        <v>0.98</v>
+        <v>10.74</v>
       </c>
       <c r="E6">
         <v>336</v>
@@ -1863,7 +1863,7 @@
         </is>
       </c>
       <c r="D7">
-        <v>1.16</v>
+        <v>10.93</v>
       </c>
       <c r="E7">
         <v>336</v>
@@ -1891,7 +1891,7 @@
         </is>
       </c>
       <c r="D8">
-        <v>0.95</v>
+        <v>10.71</v>
       </c>
       <c r="E8">
         <v>336</v>
@@ -1919,7 +1919,7 @@
         </is>
       </c>
       <c r="D9">
-        <v>0.84</v>
+        <v>10.61</v>
       </c>
       <c r="E9">
         <v>336</v>
@@ -1947,7 +1947,7 @@
         </is>
       </c>
       <c r="D10">
-        <v>1.22</v>
+        <v>10.98</v>
       </c>
       <c r="E10">
         <v>720</v>
@@ -1975,7 +1975,7 @@
         </is>
       </c>
       <c r="D11">
-        <v>0.92</v>
+        <v>0.49</v>
       </c>
       <c r="E11">
         <v>168</v>
@@ -2003,7 +2003,7 @@
         </is>
       </c>
       <c r="D12">
-        <v>2.19</v>
+        <v>0.15</v>
       </c>
       <c r="E12">
         <v>36</v>
@@ -2031,7 +2031,7 @@
         </is>
       </c>
       <c r="D13">
-        <v>11.85</v>
+        <v>21.61</v>
       </c>
       <c r="E13">
         <v>6</v>
@@ -2059,7 +2059,7 @@
         </is>
       </c>
       <c r="D14">
-        <v>1.26</v>
+        <v>0.04</v>
       </c>
       <c r="E14">
         <v>36</v>
@@ -2087,7 +2087,7 @@
         </is>
       </c>
       <c r="D15">
-        <v>0.33</v>
+        <v>0.01</v>
       </c>
       <c r="E15">
         <v>24</v>
@@ -2209,7 +2209,7 @@
         </is>
       </c>
       <c r="B6">
-        <v>1790569118</v>
+        <v>1790604240</v>
       </c>
     </row>
     <row r="7">

</xml_diff>